<commit_message>
test Data Repo : --> chargerDossier en attente validation --> test_parCTNetAnnee TODO --> test_parCodeNAF TODO --> test_parCodeNAF2 TODO --> test_rechercherActivite
</commit_message>
<xml_diff>
--- a/project/src/test/resources/2023.xlsx
+++ b/project/src/test/resources/2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rapht\Documents\IDMC\M1\Genie_Log\project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DADE8E38-231F-44C6-B73F-1FCB2AABE79A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C41D6E-D46F-4604-A74A-47ABD7B701A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6C846424-652C-4953-A543-6B556BF054B7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="49">
   <si>
     <t>AA</t>
   </si>
@@ -180,6 +180,9 @@
   </si>
   <si>
     <t>fait l'objet d'une fiche de sinistralité 2023</t>
+  </si>
+  <si>
+    <t>AB</t>
   </si>
 </sst>
 </file>
@@ -188,9 +191,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0\ _€_-;\-* #,##0\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0\ _€_-;\-* #,##0\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -333,38 +336,40 @@
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="5" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="7" fillId="3" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -702,8 +707,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B2D1A60-B977-4D30-95C3-F215F688A850}">
-  <dimension ref="A1:AG7"/>
+  <dimension ref="A1:AG8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="52.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
@@ -775,119 +783,119 @@
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
       <c r="T3" s="6"/>
-      <c r="U3" s="8" t="s">
+      <c r="U3" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="V3" s="8"/>
-      <c r="W3" s="8"/>
-      <c r="X3" s="8"/>
-      <c r="Y3" s="8"/>
-      <c r="Z3" s="8"/>
-      <c r="AA3" s="8"/>
-      <c r="AB3" s="8"/>
-      <c r="AC3" s="8"/>
-      <c r="AD3" s="8"/>
-      <c r="AE3" s="8"/>
-      <c r="AF3" s="8"/>
+      <c r="V3" s="13"/>
+      <c r="W3" s="13"/>
+      <c r="X3" s="13"/>
+      <c r="Y3" s="13"/>
+      <c r="Z3" s="13"/>
+      <c r="AA3" s="13"/>
+      <c r="AB3" s="13"/>
+      <c r="AC3" s="13"/>
+      <c r="AD3" s="13"/>
+      <c r="AE3" s="13"/>
+      <c r="AF3" s="13"/>
     </row>
     <row r="4" spans="1:33" ht="51" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="10" t="s">
+      <c r="K4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="L4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="M4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="N4" s="10" t="s">
+      <c r="N4" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="11" t="s">
+      <c r="O4" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="11" t="s">
+      <c r="P4" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="Q4" s="10" t="s">
+      <c r="Q4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="R4" s="10" t="s">
+      <c r="R4" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="S4" s="10" t="s">
+      <c r="S4" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="T4" s="10" t="s">
+      <c r="T4" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="U4" s="10" t="s">
+      <c r="U4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="V4" s="12" t="s">
+      <c r="V4" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="W4" s="10" t="s">
+      <c r="W4" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="X4" s="10" t="s">
+      <c r="X4" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="Y4" s="10" t="s">
+      <c r="Y4" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="Z4" s="10" t="s">
+      <c r="Z4" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="AA4" s="10" t="s">
+      <c r="AA4" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="AB4" s="10" t="s">
+      <c r="AB4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="AC4" s="10" t="s">
+      <c r="AC4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="AD4" s="10" t="s">
+      <c r="AD4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="AE4" s="10" t="s">
+      <c r="AE4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="AF4" s="10" t="s">
+      <c r="AF4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="AG4" s="13" t="s">
+      <c r="AG4" s="12" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1091,7 +1099,7 @@
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>1</v>
@@ -1187,6 +1195,15 @@
         <v>0</v>
       </c>
       <c r="AG7" s="4"/>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A8" s="14"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>